<commit_message>
Updated the Pivot Sheet
</commit_message>
<xml_diff>
--- a/MovieSalesDashboard.xlsx
+++ b/MovieSalesDashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04F592B9-FDC7-48DC-94B2-AFCD0DAC7C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB33616F-0897-4528-933D-59961578ADAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView showHorizontalScroll="0" showVerticalScroll="0" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{BAD933FD-3DAB-436E-B0C6-8BD739AA5275}"/>
   </bookViews>
@@ -25,7 +25,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="104" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -432,8 +432,8 @@
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    <numFmt numFmtId="175" formatCode="\$#,##0.00\ &quot;B&quot;"/>
+    <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0.00\ &quot;B&quot;"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -925,7 +925,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -934,11 +934,14 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -985,7 +988,7 @@
     <cellStyle name="Total" xfId="18" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="15" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="249">
+  <dxfs count="243">
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -993,7 +996,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1008,16 +1011,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1026,13 +1029,13 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1041,7 +1044,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1056,16 +1059,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1074,13 +1077,13 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1089,7 +1092,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1104,16 +1107,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1122,13 +1125,13 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1137,7 +1140,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1152,16 +1155,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1170,13 +1173,13 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1185,7 +1188,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1200,16 +1203,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1218,13 +1221,13 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1233,7 +1236,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1248,16 +1251,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1266,13 +1269,13 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1281,7 +1284,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1296,16 +1299,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1314,13 +1317,13 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1329,7 +1332,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1344,16 +1347,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1362,13 +1365,13 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1377,7 +1380,7 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1392,16 +1395,16 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1410,31 +1413,46 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1443,28 +1461,46 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1473,58 +1509,157 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <font>
@@ -1537,13 +1672,31 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
@@ -1552,193 +1705,25 @@
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="\$#,##0.00\ &quot;M&quot;"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="\$#,##0.00\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0,,\ &quot;M&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="#,##0,,\ &quot;M&quot;\ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="#,##0,,\ &quot;M&quot;\ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.0_ ;_-[$$-409]* \-#,##0.0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4125,6 +4110,23 @@
       <c:pivotFmt>
         <c:idx val="6"/>
         <c:spPr>
+          <a:gradFill rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:schemeClr val="accent1">
+                  <a:tint val="98000"/>
+                  <a:lumMod val="114000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:schemeClr val="accent1">
+                  <a:shade val="90000"/>
+                  <a:lumMod val="84000"/>
+                </a:schemeClr>
+              </a:gs>
+            </a:gsLst>
+            <a:lin ang="5400000" scaled="0"/>
+          </a:gradFill>
           <a:ln w="34925" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -4138,6 +4140,15 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="tl"/>
+          </a:scene3d>
+          <a:sp3d prstMaterial="plastic">
+            <a:bevelT w="0" h="0"/>
+          </a:sp3d>
         </c:spPr>
         <c:marker>
           <c:symbol val="circle"/>
@@ -11016,7 +11027,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>394607</xdr:colOff>
+      <xdr:colOff>612321</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>61233</xdr:rowOff>
     </xdr:to>
@@ -11034,7 +11045,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3088822" y="1612447"/>
-          <a:ext cx="1387928" cy="489857"/>
+          <a:ext cx="1605642" cy="489857"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -11097,16 +11108,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>84364</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>653143</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>183697</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>111578</xdr:colOff>
+      <xdr:colOff>394606</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>61233</xdr:rowOff>
+      <xdr:rowOff>136072</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="'Pivot Sheet'!I49">
       <xdr:nvSpPr>
@@ -11121,8 +11132,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7568293" y="1612447"/>
-          <a:ext cx="1387928" cy="489857"/>
+          <a:off x="7456714" y="1612447"/>
+          <a:ext cx="1782535" cy="564696"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -11151,7 +11162,7 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:fld id="{DF4B4B95-F26C-4A7C-A305-7A3DF79EF729}" type="TxLink">
-            <a:rPr lang="en-US" sz="2800" b="1" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -11167,7 +11178,7 @@
             <a:pPr algn="ctr"/>
             <a:t>4.74</a:t>
           </a:fld>
-          <a:endParaRPr lang="en-US" sz="1100" b="1">
+          <a:endParaRPr lang="en-US" sz="1200" b="1">
             <a:solidFill>
               <a:schemeClr val="bg1"/>
             </a:solidFill>
@@ -11195,7 +11206,7 @@
       <xdr:col>16</xdr:col>
       <xdr:colOff>612322</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>108858</xdr:rowOff>
+      <xdr:rowOff>163286</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="'Pivot Sheet'!D52">
       <xdr:nvSpPr>
@@ -11211,7 +11222,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9715500" y="1564822"/>
-          <a:ext cx="1782536" cy="585107"/>
+          <a:ext cx="1782536" cy="639535"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -11239,7 +11250,7 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:fld id="{2928E1FB-1BF1-41E8-9D1A-4A808F540719}" type="TxLink">
-            <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="1400" b="1" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -11252,6 +11263,7 @@
               </a:effectLst>
               <a:latin typeface="Century Gothic"/>
             </a:rPr>
+            <a:pPr algn="ctr"/>
             <a:t>The Twilight Saga: New Moon</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="1100" b="1">
@@ -12263,6 +12275,7 @@
               </a:effectLst>
               <a:latin typeface="Century Gothic"/>
             </a:rPr>
+            <a:pPr algn="ctr"/>
             <a:t>Comedy</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="1600" b="1">
@@ -12353,6 +12366,7 @@
               </a:effectLst>
               <a:latin typeface="Century Gothic"/>
             </a:rPr>
+            <a:pPr algn="ctr"/>
             <a:t>Warner Bros.</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="1400" b="1" i="0">
@@ -12386,7 +12400,7 @@
       <xdr:col>20</xdr:col>
       <xdr:colOff>108857</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>95251</xdr:rowOff>
+      <xdr:rowOff>149679</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="'Pivot Sheet'!I50">
       <xdr:nvSpPr>
@@ -12402,7 +12416,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="11906250" y="1578429"/>
-          <a:ext cx="1809750" cy="557893"/>
+          <a:ext cx="1809750" cy="612321"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -12443,6 +12457,7 @@
               </a:effectLst>
               <a:latin typeface="Century Gothic"/>
             </a:rPr>
+            <a:pPr algn="ctr"/>
             <a:t>Fireproof</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="1100" b="1" i="0" u="none" strike="noStrike">
@@ -12543,7 +12558,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="HP" refreshedDate="46138.534451041669" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="74" xr:uid="{5C259F35-FFFB-4CD0-8F4F-7ADE80AFC3C3}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="HP" refreshedDate="46138.995975810183" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="74" xr:uid="{5C259F35-FFFB-4CD0-8F4F-7ADE80AFC3C3}">
   <cacheSource type="worksheet">
     <worksheetSource name="Table1"/>
   </cacheSource>
@@ -13587,7 +13602,752 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B39BD43A-1C7E-4528-A919-C3766335D4C2}" name="PivotTable2" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5F538B46-7F88-4492-9EE7-9E15672769DF}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="21">
+  <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="14">
+        <item x="8"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="12"/>
+        <item x="3"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="1" baseItem="1" numFmtId="165"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="228">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="227">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="18" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5DCFC007-A10D-45DE-929D-BE5CC2D07F95}" name="PivotTable11" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A49:B124" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="75">
+        <item x="7"/>
+        <item x="16"/>
+        <item x="68"/>
+        <item x="20"/>
+        <item x="67"/>
+        <item x="19"/>
+        <item x="18"/>
+        <item x="22"/>
+        <item x="0"/>
+        <item x="47"/>
+        <item x="46"/>
+        <item x="15"/>
+        <item x="62"/>
+        <item x="41"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="61"/>
+        <item x="35"/>
+        <item x="71"/>
+        <item x="52"/>
+        <item x="63"/>
+        <item x="11"/>
+        <item x="57"/>
+        <item x="36"/>
+        <item x="50"/>
+        <item x="39"/>
+        <item x="51"/>
+        <item x="48"/>
+        <item x="34"/>
+        <item x="5"/>
+        <item x="23"/>
+        <item x="6"/>
+        <item x="69"/>
+        <item x="49"/>
+        <item x="26"/>
+        <item x="66"/>
+        <item x="38"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="43"/>
+        <item x="25"/>
+        <item x="72"/>
+        <item x="45"/>
+        <item x="17"/>
+        <item x="59"/>
+        <item x="58"/>
+        <item x="27"/>
+        <item x="9"/>
+        <item x="33"/>
+        <item x="40"/>
+        <item x="56"/>
+        <item x="60"/>
+        <item x="42"/>
+        <item x="53"/>
+        <item x="30"/>
+        <item x="44"/>
+        <item x="54"/>
+        <item x="8"/>
+        <item x="37"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="24"/>
+        <item x="21"/>
+        <item x="70"/>
+        <item x="3"/>
+        <item x="32"/>
+        <item x="31"/>
+        <item x="13"/>
+        <item x="73"/>
+        <item x="64"/>
+        <item x="65"/>
+        <item x="55"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="14">
+        <item x="8"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="12"/>
+        <item x="3"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="75">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i>
+      <x v="35"/>
+    </i>
+    <i>
+      <x v="36"/>
+    </i>
+    <i>
+      <x v="37"/>
+    </i>
+    <i>
+      <x v="38"/>
+    </i>
+    <i>
+      <x v="39"/>
+    </i>
+    <i>
+      <x v="40"/>
+    </i>
+    <i>
+      <x v="41"/>
+    </i>
+    <i>
+      <x v="42"/>
+    </i>
+    <i>
+      <x v="43"/>
+    </i>
+    <i>
+      <x v="44"/>
+    </i>
+    <i>
+      <x v="45"/>
+    </i>
+    <i>
+      <x v="46"/>
+    </i>
+    <i>
+      <x v="47"/>
+    </i>
+    <i>
+      <x v="48"/>
+    </i>
+    <i>
+      <x v="49"/>
+    </i>
+    <i>
+      <x v="50"/>
+    </i>
+    <i>
+      <x v="51"/>
+    </i>
+    <i>
+      <x v="52"/>
+    </i>
+    <i>
+      <x v="53"/>
+    </i>
+    <i>
+      <x v="54"/>
+    </i>
+    <i>
+      <x v="55"/>
+    </i>
+    <i>
+      <x v="56"/>
+    </i>
+    <i>
+      <x v="57"/>
+    </i>
+    <i>
+      <x v="58"/>
+    </i>
+    <i>
+      <x v="59"/>
+    </i>
+    <i>
+      <x v="60"/>
+    </i>
+    <i>
+      <x v="61"/>
+    </i>
+    <i>
+      <x v="62"/>
+    </i>
+    <i>
+      <x v="63"/>
+    </i>
+    <i>
+      <x v="64"/>
+    </i>
+    <i>
+      <x v="65"/>
+    </i>
+    <i>
+      <x v="66"/>
+    </i>
+    <i>
+      <x v="67"/>
+    </i>
+    <i>
+      <x v="68"/>
+    </i>
+    <i>
+      <x v="69"/>
+    </i>
+    <i>
+      <x v="70"/>
+    </i>
+    <i>
+      <x v="71"/>
+    </i>
+    <i>
+      <x v="72"/>
+    </i>
+    <i>
+      <x v="73"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="0" baseItem="1" numFmtId="165"/>
+  </dataFields>
+  <formats count="3">
+    <format dxfId="231">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="230">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="229">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0DC96FB9-5B51-43BB-9439-4957BE1EB5C4}" name="PivotTable16" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="66">
+  <location ref="D35:E42" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="14">
+        <item x="8"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="12"/>
+        <item x="3"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Profitability" fld="4" subtotal="average" baseField="7" baseItem="0" numFmtId="2"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="232">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="10">
+    <chartFormat chart="46" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="51" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="52" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="61" format="8" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="61" format="9">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="61" format="10">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="61" format="11">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="61" format="12">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="61" format="13">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="61" format="14">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B39BD43A-1C7E-4528-A919-C3766335D4C2}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
   <location ref="G26:H37" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0" measureFilter="1" sortType="ascending">
@@ -13773,10 +14533,10 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="0" baseItem="0" numFmtId="169"/>
+    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="187">
+    <format dxfId="235">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="1">
@@ -13785,10 +14545,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="188">
+    <format dxfId="234">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="189">
+    <format dxfId="233">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -13830,12 +14590,12 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5F538B46-7F88-4492-9EE7-9E15672769DF}" name="PivotTable1" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="21">
-  <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D2B6AF8-704C-4AF9-AF3E-D186092DA91C}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="47">
+  <location ref="A26:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0">
       <items count="7">
         <item x="5"/>
         <item x="3"/>
@@ -13847,6 +14607,130 @@
       </items>
     </pivotField>
     <pivotField showAll="0">
+      <items count="14">
+        <item x="8"/>
+        <item x="10"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="12"/>
+        <item x="3"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="7" baseItem="1" numFmtId="165"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="237">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="236">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="39" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2D10C145-7C64-4DE3-9DAC-420270FE9135}" name="PivotTable15" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="21">
+  <location ref="D3:E17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
       <items count="14">
         <item x="8"/>
         <item x="10"/>
@@ -13889,9 +14773,9 @@
     </pivotField>
   </pivotFields>
   <rowFields count="1">
-    <field x="1"/>
+    <field x="2"/>
   </rowFields>
-  <rowItems count="7">
+  <rowItems count="14">
     <i>
       <x/>
     </i>
@@ -13909,6 +14793,27 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
     </i>
     <i t="grand">
       <x/>
@@ -13918,13 +14823,13 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="1" baseItem="1" numFmtId="169"/>
+    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="2" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="216">
+    <format dxfId="239">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="174">
+    <format dxfId="238">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -13934,17 +14839,6 @@
       </pivotArea>
     </format>
   </formats>
-  <chartFormats count="1">
-    <chartFormat chart="18" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -13957,8 +14851,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A982481A-0A18-42C4-8B0B-125CA6C16EA3}" name="PivotTable12" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="53">
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A982481A-0A18-42C4-8B0B-125CA6C16EA3}" name="PivotTable12" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="53">
   <location ref="E49:F124" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0" sortType="descending">
@@ -14339,7 +15233,7 @@
     <dataField name="Sum of Profitability" fld="4" baseField="0" baseItem="18" numFmtId="2"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="215">
+    <format dxfId="240">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -14411,89 +15305,11 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5DCFC007-A10D-45DE-929D-BE5CC2D07F95}" name="PivotTable11" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A49:B124" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B8EF6DDD-8B21-4F55-A982-43B2DB6A26B6}" name="PivotTable14" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="52">
+  <location ref="D26:E32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="75">
-        <item x="7"/>
-        <item x="16"/>
-        <item x="68"/>
-        <item x="20"/>
-        <item x="67"/>
-        <item x="19"/>
-        <item x="18"/>
-        <item x="22"/>
-        <item x="0"/>
-        <item x="47"/>
-        <item x="46"/>
-        <item x="15"/>
-        <item x="62"/>
-        <item x="41"/>
-        <item x="10"/>
-        <item x="1"/>
-        <item x="61"/>
-        <item x="35"/>
-        <item x="71"/>
-        <item x="52"/>
-        <item x="63"/>
-        <item x="11"/>
-        <item x="57"/>
-        <item x="36"/>
-        <item x="50"/>
-        <item x="39"/>
-        <item x="51"/>
-        <item x="48"/>
-        <item x="34"/>
-        <item x="5"/>
-        <item x="23"/>
-        <item x="6"/>
-        <item x="69"/>
-        <item x="49"/>
-        <item x="26"/>
-        <item x="66"/>
-        <item x="38"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="43"/>
-        <item x="25"/>
-        <item x="72"/>
-        <item x="45"/>
-        <item x="17"/>
-        <item x="59"/>
-        <item x="58"/>
-        <item x="27"/>
-        <item x="9"/>
-        <item x="33"/>
-        <item x="40"/>
-        <item x="56"/>
-        <item x="60"/>
-        <item x="42"/>
-        <item x="53"/>
-        <item x="30"/>
-        <item x="44"/>
-        <item x="54"/>
-        <item x="8"/>
-        <item x="37"/>
-        <item x="2"/>
-        <item x="14"/>
-        <item x="4"/>
-        <item x="12"/>
-        <item x="24"/>
-        <item x="21"/>
-        <item x="70"/>
-        <item x="3"/>
-        <item x="32"/>
-        <item x="31"/>
-        <item x="13"/>
-        <item x="73"/>
-        <item x="64"/>
-        <item x="65"/>
-        <item x="55"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="7">
         <item x="5"/>
@@ -14524,10 +15340,10 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
+    <pivotField axis="axisRow" showAll="0">
       <items count="6">
         <item x="2"/>
         <item x="0"/>
@@ -14548,9 +15364,9 @@
     </pivotField>
   </pivotFields>
   <rowFields count="1">
-    <field x="0"/>
+    <field x="7"/>
   </rowFields>
-  <rowItems count="75">
+  <rowItems count="6">
     <i>
       <x/>
     </i>
@@ -14565,213 +15381,6 @@
     </i>
     <i>
       <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="20"/>
-    </i>
-    <i>
-      <x v="21"/>
-    </i>
-    <i>
-      <x v="22"/>
-    </i>
-    <i>
-      <x v="23"/>
-    </i>
-    <i>
-      <x v="24"/>
-    </i>
-    <i>
-      <x v="25"/>
-    </i>
-    <i>
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="30"/>
-    </i>
-    <i>
-      <x v="31"/>
-    </i>
-    <i>
-      <x v="32"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i>
-      <x v="34"/>
-    </i>
-    <i>
-      <x v="35"/>
-    </i>
-    <i>
-      <x v="36"/>
-    </i>
-    <i>
-      <x v="37"/>
-    </i>
-    <i>
-      <x v="38"/>
-    </i>
-    <i>
-      <x v="39"/>
-    </i>
-    <i>
-      <x v="40"/>
-    </i>
-    <i>
-      <x v="41"/>
-    </i>
-    <i>
-      <x v="42"/>
-    </i>
-    <i>
-      <x v="43"/>
-    </i>
-    <i>
-      <x v="44"/>
-    </i>
-    <i>
-      <x v="45"/>
-    </i>
-    <i>
-      <x v="46"/>
-    </i>
-    <i>
-      <x v="47"/>
-    </i>
-    <i>
-      <x v="48"/>
-    </i>
-    <i>
-      <x v="49"/>
-    </i>
-    <i>
-      <x v="50"/>
-    </i>
-    <i>
-      <x v="51"/>
-    </i>
-    <i>
-      <x v="52"/>
-    </i>
-    <i>
-      <x v="53"/>
-    </i>
-    <i>
-      <x v="54"/>
-    </i>
-    <i>
-      <x v="55"/>
-    </i>
-    <i>
-      <x v="56"/>
-    </i>
-    <i>
-      <x v="57"/>
-    </i>
-    <i>
-      <x v="58"/>
-    </i>
-    <i>
-      <x v="59"/>
-    </i>
-    <i>
-      <x v="60"/>
-    </i>
-    <i>
-      <x v="61"/>
-    </i>
-    <i>
-      <x v="62"/>
-    </i>
-    <i>
-      <x v="63"/>
-    </i>
-    <i>
-      <x v="64"/>
-    </i>
-    <i>
-      <x v="65"/>
-    </i>
-    <i>
-      <x v="66"/>
-    </i>
-    <i>
-      <x v="67"/>
-    </i>
-    <i>
-      <x v="68"/>
-    </i>
-    <i>
-      <x v="69"/>
-    </i>
-    <i>
-      <x v="70"/>
-    </i>
-    <i>
-      <x v="71"/>
-    </i>
-    <i>
-      <x v="72"/>
-    </i>
-    <i>
-      <x v="73"/>
     </i>
     <i t="grand">
       <x/>
@@ -14781,25 +15390,24 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="0" baseItem="1" numFmtId="169"/>
+    <dataField name="Average of Profitability" fld="4" subtotal="average" baseField="7" baseItem="0" numFmtId="2"/>
   </dataFields>
-  <formats count="3">
-    <format dxfId="213">
+  <formats count="1">
+    <format dxfId="241">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="214">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="167">
-      <pivotArea outline="0" fieldPosition="0">
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="51" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
         </references>
       </pivotArea>
-    </format>
-  </formats>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -14812,8 +15420,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72FFCFC2-5C82-4228-B308-39CE0CF887B7}" name="PivotTable10" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="53">
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72FFCFC2-5C82-4228-B308-39CE0CF887B7}" name="PivotTable10" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="53">
   <location ref="A35:B46" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0" measureFilter="1" sortType="ascending">
@@ -15002,7 +15610,7 @@
     <dataField name="Average of Profitability" fld="4" subtotal="average" baseField="7" baseItem="2" numFmtId="2"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="212">
+    <format dxfId="242">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -15063,599 +15671,6 @@
       </autoFilter>
     </filter>
   </filters>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0DC96FB9-5B51-43BB-9439-4957BE1EB5C4}" name="PivotTable16" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="66">
-  <location ref="D35:E42" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="14">
-        <item x="8"/>
-        <item x="10"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="7"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item x="12"/>
-        <item x="3"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Profitability" fld="4" subtotal="average" baseField="7" baseItem="0" numFmtId="2"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="211">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="10">
-    <chartFormat chart="46" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="51" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="52" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="61" format="8" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="61" format="9">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="61" format="10">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="61" format="11">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="61" format="12">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="61" format="13">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="61" format="14">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2D10C145-7C64-4DE3-9DAC-420270FE9135}" name="PivotTable15" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="21">
-  <location ref="D3:E17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="14">
-        <item x="8"/>
-        <item x="10"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="7"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item x="12"/>
-        <item x="3"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="2" baseItem="0" numFmtId="169"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="210">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="171">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D2B6AF8-704C-4AF9-AF3E-D186092DA91C}" name="PivotTable7" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="47">
-  <location ref="A26:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="14">
-        <item x="8"/>
-        <item x="10"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="7"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item x="12"/>
-        <item x="3"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Worldwide Gross($M)" fld="6" baseField="7" baseItem="1" numFmtId="169"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="209">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="178">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="39" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B8EF6DDD-8B21-4F55-A982-43B2DB6A26B6}" name="PivotTable14" cacheId="104" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="52">
-  <location ref="D26:E32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="14">
-        <item x="8"/>
-        <item x="10"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="7"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item x="12"/>
-        <item x="3"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Profitability" fld="4" subtotal="average" baseField="7" baseItem="0" numFmtId="2"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="208">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="51" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
@@ -15806,10 +15821,10 @@
     <tableColumn id="6" xr3:uid="{8EAF23C7-2A06-4D3E-85D8-068C05E92791}" name="Rotten Tomatoes %"/>
     <tableColumn id="7" xr3:uid="{F3633C84-0170-4F69-955D-D9E079290AF0}" name="Worldwide Gross($M)"/>
     <tableColumn id="8" xr3:uid="{FDD3A7B5-16A3-4821-8C7E-9581399648D6}" name="Year"/>
-    <tableColumn id="9" xr3:uid="{0FDED1A2-64C3-4741-98C2-BBDF12607A2B}" name="Combined Score" dataDxfId="248">
+    <tableColumn id="9" xr3:uid="{0FDED1A2-64C3-4741-98C2-BBDF12607A2B}" name="Combined Score" dataDxfId="226">
       <calculatedColumnFormula>(Table1[[#This Row],[Audience  score %]]+Table1[[#This Row],[Rotten Tomatoes %]])/2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{B3A5B06A-87D9-465B-ADDF-C1F00620126C}" name="Rating Level" dataDxfId="247">
+    <tableColumn id="10" xr3:uid="{B3A5B06A-87D9-465B-ADDF-C1F00620126C}" name="Rating Level" dataDxfId="225">
       <calculatedColumnFormula>IF(Table1[[#This Row],[Combined Score]]&gt;=75,"High",IF(Table1[[#This Row],[Combined Score]]&gt;40,"Medium","Low"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -16128,12 +16143,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="7"/>
+      <c r="B2" s="9"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>101</v>
       </c>
@@ -16149,8 +16164,17 @@
       <c r="G3" t="s">
         <v>110</v>
       </c>
-      <c r="H3" t="str" cm="1">
-        <f t="array" ref="H3">_xlfn._xlws.FILTER(D4:D16, E4:E16=MAX(E4:E16))</f>
+      <c r="H3" s="8" t="str" cm="1">
+        <f t="array" ref="H3">IFERROR(
+   INDEX(D4:D16,
+      MATCH(
+         MAX(IF((D4:D16&lt;&gt;"Grand Total")*(E4:E16&lt;&gt;""),E4:E16)),
+         E4:E16,
+         0
+      )
+   ),
+   "-"
+)</f>
         <v>Warner Bros.</v>
       </c>
     </row>
@@ -16168,6 +16192,16 @@
       <c r="E4" s="6">
         <v>156.75799999999998</v>
       </c>
+      <c r="H4" s="8" t="str" cm="1">
+        <f t="array" ref="H4">IFERROR(INDEX(D5:D17,
+MATCH(
+MAX(IF(D5:D17&lt;&gt;"Grand Total",E5:E17)),
+E5:E17,
+0
+)
+),"-")</f>
+        <v>Warner Bros.</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -16184,7 +16218,7 @@
         <v>77.09</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -16201,8 +16235,14 @@
       <c r="G6" t="s">
         <v>111</v>
       </c>
-      <c r="H6" t="str" cm="1">
-        <f t="array" ref="H6">_xlfn._xlws.FILTER(A4:A9,B4:B9=MAX(B4:B9))</f>
+      <c r="H6" s="8" t="str" cm="1">
+        <f t="array" ref="H6">IFERROR(INDEX(A4:A9,
+ MATCH(
+   MAX(IF(A4:A9&lt;&gt;"Grand Total", B4:B9)),
+   B4:B9,
+   0
+ )
+),"-")</f>
         <v>Comedy</v>
       </c>
     </row>
@@ -16696,7 +16736,7 @@
         <v>108</v>
       </c>
       <c r="I49" s="4">
-        <f>AVERAGE(F50:F120)</f>
+        <f>IF(COUNTA(F50:F120)=0, "-", AVERAGE(F50:F120))</f>
         <v>4.741609796577464</v>
       </c>
     </row>
@@ -16710,7 +16750,7 @@
       <c r="C50" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D50" s="8">
+      <c r="D50" s="7">
         <f>SUM(B50:B123)/1000</f>
         <v>10.09004644</v>
       </c>
@@ -16724,7 +16764,13 @@
         <v>113</v>
       </c>
       <c r="I50" t="str" cm="1">
-        <f t="array" ref="I50">_xlfn._xlws.FILTER(E50:E123, F50:F123=MAX(F50:F123))</f>
+        <f t="array" ref="I50">IFERROR(INDEX(E50:E122,
+MATCH(
+MAX(IF(E50:E122&lt;&gt;"Grand Total",F50:F122)),
+F50:F122,
+0
+)
+),"-")</f>
         <v>Fireproof</v>
       </c>
     </row>
@@ -16739,7 +16785,7 @@
         <v>105</v>
       </c>
       <c r="D51">
-        <f>COUNTA(A50:A123)</f>
+        <f>MAX(0,SUBTOTAL(3,A50:A124)-1)</f>
         <v>74</v>
       </c>
       <c r="E51" s="2" t="s">
@@ -16760,7 +16806,11 @@
         <v>112</v>
       </c>
       <c r="D52" t="str" cm="1">
-        <f t="array" ref="D52">_xlfn._xlws.FILTER(A50:A123,B50:B123=MAX(B50:B123))</f>
+        <f t="array" ref="D52">IF(SUBTOTAL(3,A50:A123)&lt;=1,"-",
+INDEX(A50:A123,
+MATCH(MAX(IF((A50:A123&lt;&gt;"Grand Total"),B50:B123)),
+B50:B123,0))
+)</f>
         <v>The Twilight Saga: New Moon</v>
       </c>
       <c r="E52" s="2" t="s">
@@ -20406,7 +20456,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="180" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="224" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>